<commit_message>
Fixed data loading and moved functions into smaller files
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Heuristic/inputData.xlsx
+++ b/Heuristic/inputData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/HanSong_Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\Heuristic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431D7377-A50A-F541-96AB-2F5AEC408954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D8BB6A-01C8-469D-A575-7A5C2484BD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16320" activeTab="3" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="54">
   <si>
     <t>type</t>
   </si>
@@ -118,15 +118,6 @@
   </si>
   <si>
     <t>(37.5176, 127.0867)</t>
-  </si>
-  <si>
-    <t>(37.6686, 126.7443)</t>
-  </si>
-  <si>
-    <t>(37.5254, 126.9215)</t>
-  </si>
-  <si>
-    <t>(37.4875, 127.1013)</t>
   </si>
   <si>
     <t>Plane ID</t>
@@ -613,7 +604,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="5"/>
@@ -621,105 +612,105 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B2" s="5">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B3" s="5">
         <v>0.75</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B4" s="5">
         <v>300</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B5" s="5">
         <v>1.51</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B6" s="5">
         <v>0.3</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B7" s="5">
         <v>0.2</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B9" s="5">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B10" s="5">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B11" s="5">
         <v>100</v>
@@ -730,7 +721,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B12" s="5">
         <v>10</v>
@@ -741,46 +732,46 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B13" s="5">
         <v>5</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B14" s="5">
         <v>6</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B15" s="5">
         <v>20</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B16" s="5">
         <v>120</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -791,7 +782,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3CF6DF-5DC6-4F82-AD2C-07BC625FD2D9}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
@@ -961,7 +952,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{332D5C3C-A1DF-48A5-A3F8-29AFDB8C103D}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -970,17 +961,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE46B-0EE8-4D7E-956E-06AD6DDE4FF5}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1023,17 +1014,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A48C4B-C23A-0343-9CD4-B20C0FE9227B}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1068,7 +1059,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="22.5" customWidth="1"/>
   </cols>
@@ -1086,6 +1077,9 @@
       <c r="D1" t="s">
         <v>4</v>
       </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
       <c r="I1" t="s">
         <v>21</v>
       </c>
@@ -1100,8 +1094,11 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>22</v>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>5</v>
@@ -1120,8 +1117,11 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
-        <v>23</v>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>6</v>
@@ -1140,8 +1140,11 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
-        <v>24</v>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>7</v>
@@ -1160,8 +1163,11 @@
       <c r="C5">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
-        <v>25</v>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>11</v>
@@ -1180,8 +1186,11 @@
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="D6" t="s">
-        <v>26</v>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>13</v>
@@ -1199,7 +1208,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
   <dimension ref="A1:X32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>
@@ -1767,7 +1776,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF01B7F4-A8F2-E74F-93E1-1ACB4B99B891}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
@@ -1837,7 +1846,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4154E97-9715-C248-8300-688A466787B4}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="12.5" customWidth="1"/>
   </cols>
@@ -1916,7 +1925,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="12.5" customWidth="1"/>
     <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
@@ -1950,8 +1959,8 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>22</v>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>5</v>
@@ -1970,8 +1979,8 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
-        <v>23</v>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>6</v>
@@ -1990,8 +1999,8 @@
       <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4" t="s">
-        <v>24</v>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>7</v>
@@ -2010,8 +2019,8 @@
       <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
-        <v>25</v>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>11</v>
@@ -2030,8 +2039,8 @@
       <c r="C6">
         <v>2</v>
       </c>
-      <c r="D6" t="s">
-        <v>26</v>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>13</v>
@@ -2049,7 +2058,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A73ABDEA-DD83-4C31-B1A2-B93032C8B1F1}">
   <dimension ref="A1:X32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>
@@ -2075,7 +2084,7 @@
         <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2090,7 +2099,7 @@
       </c>
       <c r="D2">
         <f ca="1">RANDBETWEEN(10,120)</f>
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -2100,15 +2109,15 @@
       </c>
       <c r="I2">
         <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2">
         <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2">
         <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -2123,7 +2132,7 @@
       </c>
       <c r="D3">
         <f t="shared" ref="D3:D21" ca="1" si="0">RANDBETWEEN(10,120)</f>
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -2133,11 +2142,11 @@
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I21" ca="1" si="1">RANDBETWEEN(1,5)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K3">
         <f t="shared" ref="K3:L21" ca="1" si="2">RANDBETWEEN(1,5)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L3">
         <f t="shared" ca="1" si="2"/>
@@ -2156,7 +2165,7 @@
       </c>
       <c r="D4">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -2166,15 +2175,15 @@
       </c>
       <c r="I4">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L4">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -2189,7 +2198,7 @@
       </c>
       <c r="D5">
         <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -2199,15 +2208,15 @@
       </c>
       <c r="I5">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L5">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -2222,7 +2231,7 @@
       </c>
       <c r="D6">
         <f t="shared" ca="1" si="0"/>
-        <v>117</v>
+        <v>43</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2232,15 +2241,15 @@
       </c>
       <c r="I6">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L6">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2255,7 +2264,7 @@
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="0"/>
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2265,15 +2274,15 @@
       </c>
       <c r="I7">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L7">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2288,7 +2297,7 @@
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2298,15 +2307,15 @@
       </c>
       <c r="I8">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L8">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2321,7 +2330,7 @@
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>16</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -2331,15 +2340,15 @@
       </c>
       <c r="I9">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K9">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2354,7 +2363,7 @@
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -2364,15 +2373,15 @@
       </c>
       <c r="I10">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L10">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2387,7 +2396,7 @@
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2401,11 +2410,11 @@
       </c>
       <c r="K11">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2420,7 +2429,7 @@
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2430,7 +2439,7 @@
       </c>
       <c r="I12">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K12">
         <f t="shared" ca="1" si="2"/>
@@ -2438,7 +2447,7 @@
       </c>
       <c r="L12">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2453,7 +2462,7 @@
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -2463,15 +2472,15 @@
       </c>
       <c r="I13">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K13">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L13">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -2486,7 +2495,7 @@
       </c>
       <c r="D14">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -2496,7 +2505,7 @@
       </c>
       <c r="I14">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14">
         <f t="shared" ca="1" si="2"/>
@@ -2519,7 +2528,7 @@
       </c>
       <c r="D15">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2529,7 +2538,7 @@
       </c>
       <c r="I15">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K15">
         <f t="shared" ca="1" si="2"/>
@@ -2537,7 +2546,7 @@
       </c>
       <c r="L15">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2552,7 +2561,7 @@
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -2562,15 +2571,15 @@
       </c>
       <c r="I16">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K16">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L16">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:24">
@@ -2585,7 +2594,7 @@
       </c>
       <c r="D17">
         <f t="shared" ca="1" si="0"/>
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="E17">
         <v>3</v>
@@ -2603,7 +2612,7 @@
       </c>
       <c r="L17">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -2618,7 +2627,7 @@
       </c>
       <c r="D18">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -2628,15 +2637,15 @@
       </c>
       <c r="I18">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L18">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -2651,7 +2660,7 @@
       </c>
       <c r="D19">
         <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2661,15 +2670,15 @@
       </c>
       <c r="I19">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K19">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:24">
@@ -2684,7 +2693,7 @@
       </c>
       <c r="D20">
         <f t="shared" ca="1" si="0"/>
-        <v>118</v>
+        <v>17</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -2698,11 +2707,11 @@
       </c>
       <c r="K20">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L20">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:24">
@@ -2717,7 +2726,7 @@
       </c>
       <c r="D21">
         <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2731,11 +2740,11 @@
       </c>
       <c r="K21">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L21">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:24">

</xml_diff>

<commit_message>
Fixed, and removed air corridor feasibility check
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Heuristic/inputData.xlsx
+++ b/Heuristic/inputData.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\Heuristic\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/HanSong_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D8BB6A-01C8-469D-A575-7A5C2484BD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8904C5-630C-4340-8F2B-69D62A7AD696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" firstSheet="1" activeTab="10" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
-    <sheet name="PlaneData" sheetId="7" r:id="rId2"/>
-    <sheet name="PlaneData (2)" sheetId="8" r:id="rId3"/>
-    <sheet name="Infrastructure" sheetId="1" r:id="rId4"/>
-    <sheet name="PassengerGroups" sheetId="2" r:id="rId5"/>
-    <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId6"/>
-    <sheet name="Infrastructure (2)" sheetId="4" r:id="rId7"/>
-    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId8"/>
-    <sheet name="PassengerGroups (4)" sheetId="11" r:id="rId9"/>
-    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId10"/>
-    <sheet name="Sheet1" sheetId="10" r:id="rId11"/>
+    <sheet name="Prices" sheetId="12" r:id="rId2"/>
+    <sheet name="PlaneData" sheetId="7" r:id="rId3"/>
+    <sheet name="PlaneData (2)" sheetId="8" r:id="rId4"/>
+    <sheet name="Infrastructure" sheetId="1" r:id="rId5"/>
+    <sheet name="PassengerGroups" sheetId="2" r:id="rId6"/>
+    <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId7"/>
+    <sheet name="Infrastructure (2)" sheetId="4" r:id="rId8"/>
+    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId9"/>
+    <sheet name="PassengerGroups (4)" sheetId="11" r:id="rId10"/>
+    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId11"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="80">
   <si>
     <t>type</t>
   </si>
@@ -120,15 +121,21 @@
     <t>(37.5176, 127.0867)</t>
   </si>
   <si>
+    <t>(37.6686, 126.7443)</t>
+  </si>
+  <si>
+    <t>(37.5254, 126.9215)</t>
+  </si>
+  <si>
+    <t>(37.4875, 127.1013)</t>
+  </si>
+  <si>
     <t>Plane ID</t>
   </si>
   <si>
     <t>Base Vertiport</t>
   </si>
   <si>
-    <t>cap_flt</t>
-  </si>
-  <si>
     <t>cap_u</t>
   </si>
   <si>
@@ -162,18 +169,9 @@
     <t>e_{i,j} = 1%/km</t>
   </si>
   <si>
-    <t>rt_{i,j} = 0.6 min/km</t>
-  </si>
-  <si>
-    <t>capacity of air corridor</t>
-  </si>
-  <si>
     <t>seat capacity of eVTOL</t>
   </si>
   <si>
-    <t>5% battery charged per unit time</t>
-  </si>
-  <si>
     <t>minimum turnaround time at vertiport</t>
   </si>
   <si>
@@ -207,14 +205,99 @@
     <t>Helper Column</t>
   </si>
   <si>
-    <t xml:space="preserve">cap_v </t>
+    <t>Bil tid (min)</t>
+  </si>
+  <si>
+    <t>Km fugleflugt</t>
+  </si>
+  <si>
+    <t>eVTOL flyvetid (min)</t>
+  </si>
+  <si>
+    <t>Hvor meget hurtigere</t>
+  </si>
+  <si>
+    <t>Fd km</t>
+  </si>
+  <si>
+    <t>Fd tid</t>
+  </si>
+  <si>
+    <t>fd max</t>
+  </si>
+  <si>
+    <t>Passager km pris</t>
+  </si>
+  <si>
+    <t>kr/km</t>
+  </si>
+  <si>
+    <t>Tidsværdi</t>
+  </si>
+  <si>
+    <t>kr/min</t>
+  </si>
+  <si>
+    <t>Lambda</t>
+  </si>
+  <si>
+    <t>Base fee</t>
+  </si>
+  <si>
+    <t>kr</t>
+  </si>
+  <si>
+    <t>From</t>
+  </si>
+  <si>
+    <t>To</t>
+  </si>
+  <si>
+    <t>fd_sum</t>
+  </si>
+  <si>
+    <t>2,1% battery charged per unit time</t>
+  </si>
+  <si>
+    <t>rt_{i,j} = 0.2 min/km</t>
+  </si>
+  <si>
+    <t>unit time</t>
+  </si>
+  <si>
+    <t>b_penalty</t>
+  </si>
+  <si>
+    <t>penalty for not serving passengergroup</t>
+  </si>
+  <si>
+    <t>penalty for exceeding bmax</t>
+  </si>
+  <si>
+    <t>bmid</t>
+  </si>
+  <si>
+    <t>opening_cost</t>
+  </si>
+  <si>
+    <t>cost of opening a vertiport</t>
+  </si>
+  <si>
+    <t>minuts/unit</t>
+  </si>
+  <si>
+    <t>time_old</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -239,6 +322,27 @@
       <color rgb="FF000000"/>
       <name val="CharisSIL"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -257,10 +361,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -269,8 +374,28 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -603,8 +728,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="5"/>
@@ -612,119 +737,126 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="5">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" s="5">
         <v>0.75</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="B4" s="5">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B5" s="5">
-        <v>1.51</v>
+        <v>300</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B6" s="5">
-        <v>0.3</v>
+        <v>1.51</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B7" s="5">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>48</v>
+      </c>
+      <c r="B8" s="5">
+        <f>0.2/B20</f>
+        <v>0.04</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B9" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B10" s="5">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
-        <v>40</v>
+        <v>100</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="B11" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D11" s="4">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B12" s="5">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D12" s="4">
         <v>0.1</v>
@@ -732,471 +864,72 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>72</v>
       </c>
       <c r="B13" s="5">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>41</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14" s="5">
-        <v>6</v>
+        <f>2.11*B20</f>
+        <v>10.549999999999999</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="5">
-        <v>20</v>
+        <f>30/B20</f>
+        <v>6</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B16" s="5">
-        <v>120</v>
+        <f>20/B20</f>
+        <v>4</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3CF6DF-5DC6-4F82-AD2C-07BC625FD2D9}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2">
-        <v>25</v>
-      </c>
-      <c r="E2">
-        <v>3</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>50</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>5</v>
-      </c>
-      <c r="D4">
-        <v>70</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>40</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>110</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
         <v>35</v>
       </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>3</v>
-      </c>
-      <c r="D8">
-        <v>45</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{332D5C3C-A1DF-48A5-A3F8-29AFDB8C103D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE46B-0EE8-4D7E-956E-06AD6DDE4FF5}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
-  <cols>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="B17" s="5">
+        <f>120/B20</f>
         <v>24</v>
       </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A48C4B-C23A-0343-9CD4-B20C0FE9227B}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
-  <cols>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
-  <cols>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K6" t="s">
-        <v>14</v>
+      <c r="D17" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5">
+        <v>5</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1205,16 +938,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A73ABDEA-DD83-4C31-B1A2-B93032C8B1F1}">
   <dimension ref="A1:X32"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1233,19 +966,23 @@
       <c r="F1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="I1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
       <c r="D2">
-        <v>45</v>
+        <f ca="1">RANDBETWEEN(10,120)</f>
+        <v>86</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1253,19 +990,32 @@
       <c r="F2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="I2">
+        <f ca="1">RANDBETWEEN(1,5)</f>
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <f ca="1">RANDBETWEEN(1,5)</f>
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <f ca="1">RANDBETWEEN(1,5)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>80</v>
+        <f t="shared" ref="D3:D21" ca="1" si="0">RANDBETWEEN(10,120)</f>
+        <v>61</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -1273,8 +1023,20 @@
       <c r="F3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="I3">
+        <f t="shared" ref="I3:I21" ca="1" si="1">RANDBETWEEN(1,5)</f>
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <f t="shared" ref="K3:L21" ca="1" si="2">RANDBETWEEN(1,5)</f>
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1282,10 +1044,11 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -1293,8 +1056,20 @@
       <c r="F4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="I4">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1305,7 +1080,8 @@
         <v>3</v>
       </c>
       <c r="D5">
-        <v>70</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>92</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -1313,19 +1089,32 @@
       <c r="F5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="I5">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>110</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>114</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -1333,19 +1122,32 @@
       <c r="F6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="I6">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <f t="shared" ca="1" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>35</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>80</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -1353,19 +1155,32 @@
       <c r="F7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="I7">
+        <f t="shared" ca="1" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8">
         <v>3</v>
       </c>
       <c r="D8">
-        <v>45</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>88</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -1373,19 +1188,32 @@
       <c r="F8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="I8">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K8">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="L8">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>60</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>94</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -1393,19 +1221,32 @@
       <c r="F9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="I9">
+        <f t="shared" ca="1" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="K9">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="L9">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10">
-        <v>40</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>102</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -1413,19 +1254,32 @@
       <c r="F10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="I10">
+        <f t="shared" ca="1" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L10">
+        <f t="shared" ca="1" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C11">
         <v>4</v>
       </c>
       <c r="D11">
-        <v>50</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>86</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -1433,19 +1287,32 @@
       <c r="F11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="I11">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <f t="shared" ca="1" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="L11">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
       <c r="D12">
-        <v>20</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>37</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1453,19 +1320,32 @@
       <c r="F12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="I12">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K12">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <f t="shared" ca="1" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D13">
-        <v>30</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>26</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -1473,19 +1353,32 @@
       <c r="F13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="I13">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="K13">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L13">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14">
-        <v>20</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>100</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -1493,19 +1386,32 @@
       <c r="F14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="I14">
+        <f t="shared" ca="1" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="K14">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="L14">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15">
-        <v>50</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>37</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -1513,25 +1419,50 @@
       <c r="F15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="I15">
+        <f t="shared" ca="1" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L15">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16">
-        <v>35</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>59</v>
       </c>
       <c r="E16">
         <v>3</v>
       </c>
       <c r="F16">
         <v>0</v>
+      </c>
+      <c r="I16">
+        <f t="shared" ca="1" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="K16">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L16">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:24">
@@ -1539,19 +1470,32 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17">
-        <v>20</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>22</v>
       </c>
       <c r="E17">
         <v>3</v>
       </c>
       <c r="F17">
         <v>1</v>
+      </c>
+      <c r="I17">
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K17">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L17">
+        <f t="shared" ca="1" si="2"/>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -1559,19 +1503,32 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18">
-        <v>65</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>111</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18">
         <v>0</v>
+      </c>
+      <c r="I18">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="K18">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L18">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -1579,19 +1536,32 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D19">
-        <v>90</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>19</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19">
         <v>0</v>
+      </c>
+      <c r="I19">
+        <f t="shared" ca="1" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="K19">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L19">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:24">
@@ -1599,19 +1569,32 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D20">
-        <v>15</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>21</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20">
         <v>0</v>
+      </c>
+      <c r="I20">
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="K20">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="L20">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:24">
@@ -1619,19 +1602,32 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21">
-        <v>60</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>24</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="F21">
         <v>0</v>
+      </c>
+      <c r="I21">
+        <f t="shared" ca="1" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="K21">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L21">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:24">
@@ -1773,12 +1769,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF01B7F4-A8F2-E74F-93E1-1ACB4B99B891}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3CF6DF-5DC6-4F82-AD2C-07BC625FD2D9}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <cols>
+    <col min="5" max="5" width="19.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1789,7 +1788,7 @@
         <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>79</v>
       </c>
       <c r="E1" t="s">
         <v>19</v>
@@ -1797,19 +1796,22 @@
       <c r="F1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1817,25 +1819,153 @@
       <c r="F2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2">
+        <f>D2/5</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="E3">
         <v>3</v>
       </c>
       <c r="F3">
         <v>0</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G8" si="0">D3/5</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>70</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>40</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>110</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>35</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>45</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1843,96 +1973,729 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4154E97-9715-C248-8300-688A466787B4}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{332D5C3C-A1DF-48A5-A3F8-29AFDB8C103D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF0D5EA-53B5-1240-9D84-6FE223856A18}">
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="3" max="3" width="12.5" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:14">
+      <c r="A1" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="N1" s="8"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10">
+        <v>2</v>
+      </c>
+      <c r="C2" s="10">
+        <f>(180)</f>
+        <v>180</v>
+      </c>
+      <c r="D2" s="10">
+        <v>219</v>
+      </c>
+      <c r="E2" s="10">
+        <f t="shared" ref="E2:E11" si="0">$M$1*D2</f>
+        <v>43.800000000000004</v>
+      </c>
+      <c r="F2" s="11">
+        <f>C2/E2</f>
+        <v>4.10958904109589</v>
+      </c>
+      <c r="G2" s="12">
+        <f t="shared" ref="G2:G11" si="1">D2*$M$2</f>
+        <v>4161</v>
+      </c>
+      <c r="H2" s="13">
+        <f t="shared" ref="H2:H11" si="2">(C2-E2)*$M$3*$M$4</f>
+        <v>1589</v>
+      </c>
+      <c r="I2" s="13">
+        <f>G2+H2</f>
+        <v>5750</v>
+      </c>
+      <c r="J2" s="13">
+        <f t="shared" ref="J2:J11" si="3">MAX($M$2*D2+$M$5,$M$4*$M$3*(C2-E2))</f>
+        <v>4161</v>
+      </c>
+      <c r="L2" t="s">
+        <v>59</v>
+      </c>
+      <c r="M2" s="5">
+        <v>19</v>
+      </c>
+      <c r="N2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10">
+        <v>3</v>
+      </c>
+      <c r="C3" s="10">
+        <v>60</v>
+      </c>
+      <c r="D3" s="10">
+        <v>88</v>
+      </c>
+      <c r="E3" s="10">
+        <f t="shared" si="0"/>
+        <v>17.600000000000001</v>
+      </c>
+      <c r="F3" s="11">
+        <f t="shared" ref="F3:F11" si="4">C3/E3</f>
+        <v>3.4090909090909087</v>
+      </c>
+      <c r="G3" s="12">
+        <f t="shared" si="1"/>
+        <v>1672</v>
+      </c>
+      <c r="H3" s="13">
+        <f t="shared" si="2"/>
+        <v>494.66666666666669</v>
+      </c>
+      <c r="I3" s="13">
+        <f t="shared" ref="I3:I11" si="5">G3+H3</f>
+        <v>2166.6666666666665</v>
+      </c>
+      <c r="J3" s="13">
+        <f t="shared" si="3"/>
+        <v>1672</v>
+      </c>
+      <c r="L3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" s="5">
+        <f>1000/60</f>
+        <v>16.666666666666668</v>
+      </c>
+      <c r="N3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10">
+        <v>4</v>
+      </c>
+      <c r="C4" s="10">
+        <f>200</f>
+        <v>200</v>
+      </c>
+      <c r="D4" s="10">
+        <v>147</v>
+      </c>
+      <c r="E4" s="10">
+        <f t="shared" si="0"/>
+        <v>29.400000000000002</v>
+      </c>
+      <c r="F4" s="11">
+        <f t="shared" si="4"/>
+        <v>6.8027210884353737</v>
+      </c>
+      <c r="G4" s="12">
+        <f t="shared" si="1"/>
+        <v>2793</v>
+      </c>
+      <c r="H4" s="13">
+        <f t="shared" si="2"/>
+        <v>1990.3333333333333</v>
+      </c>
+      <c r="I4" s="13">
+        <f t="shared" si="5"/>
+        <v>4783.333333333333</v>
+      </c>
+      <c r="J4" s="13">
+        <f t="shared" si="3"/>
+        <v>2793</v>
+      </c>
+      <c r="L4" t="s">
+        <v>63</v>
+      </c>
+      <c r="M4" s="5">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="10">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10">
+        <f>(60+50)</f>
+        <v>110</v>
+      </c>
+      <c r="D5" s="10">
+        <v>147</v>
+      </c>
+      <c r="E5" s="10">
+        <f t="shared" si="0"/>
+        <v>29.400000000000002</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" si="4"/>
+        <v>3.7414965986394555</v>
+      </c>
+      <c r="G5" s="12">
+        <f t="shared" si="1"/>
+        <v>2793</v>
+      </c>
+      <c r="H5" s="13">
+        <f t="shared" si="2"/>
+        <v>940.33333333333326</v>
+      </c>
+      <c r="I5" s="13">
+        <f t="shared" si="5"/>
+        <v>3733.333333333333</v>
+      </c>
+      <c r="J5" s="13">
+        <f t="shared" si="3"/>
+        <v>2793</v>
+      </c>
+      <c r="L5" t="s">
+        <v>64</v>
+      </c>
+      <c r="M5" s="5">
+        <v>0</v>
+      </c>
+      <c r="N5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" s="10">
+        <v>3</v>
+      </c>
+      <c r="C6" s="10">
+        <f>(120+40)</f>
+        <v>160</v>
+      </c>
+      <c r="D6" s="10">
+        <v>131</v>
+      </c>
+      <c r="E6" s="10">
+        <f t="shared" si="0"/>
+        <v>26.200000000000003</v>
+      </c>
+      <c r="F6" s="11">
+        <f t="shared" si="4"/>
+        <v>6.1068702290076331</v>
+      </c>
+      <c r="G6" s="12">
+        <f t="shared" si="1"/>
+        <v>2489</v>
+      </c>
+      <c r="H6" s="13">
+        <f t="shared" si="2"/>
+        <v>1561.0000000000002</v>
+      </c>
+      <c r="I6" s="13">
+        <f t="shared" si="5"/>
+        <v>4050</v>
+      </c>
+      <c r="J6" s="13">
+        <f t="shared" si="3"/>
+        <v>2489</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" s="10">
+        <v>4</v>
+      </c>
+      <c r="C7" s="10">
+        <f>90</f>
+        <v>90</v>
+      </c>
+      <c r="D7" s="10">
+        <v>111</v>
+      </c>
+      <c r="E7" s="10">
+        <f t="shared" si="0"/>
+        <v>22.200000000000003</v>
+      </c>
+      <c r="F7" s="11">
+        <f t="shared" si="4"/>
+        <v>4.0540540540540535</v>
+      </c>
+      <c r="G7" s="12">
+        <f t="shared" si="1"/>
+        <v>2109</v>
+      </c>
+      <c r="H7" s="13">
+        <f t="shared" si="2"/>
+        <v>791</v>
+      </c>
+      <c r="I7" s="13">
+        <f t="shared" si="5"/>
+        <v>2900</v>
+      </c>
+      <c r="J7" s="13">
+        <f t="shared" si="3"/>
+        <v>2109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" s="10">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10">
+        <f>75</f>
+        <v>75</v>
+      </c>
+      <c r="D8" s="10">
+        <v>80</v>
+      </c>
+      <c r="E8" s="10">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="F8" s="11">
+        <f t="shared" si="4"/>
+        <v>4.6875</v>
+      </c>
+      <c r="G8" s="12">
+        <f t="shared" si="1"/>
+        <v>1520</v>
+      </c>
+      <c r="H8" s="13">
+        <f t="shared" si="2"/>
+        <v>688.33333333333337</v>
+      </c>
+      <c r="I8" s="13">
+        <f t="shared" si="5"/>
+        <v>2208.3333333333335</v>
+      </c>
+      <c r="J8" s="13">
+        <f t="shared" si="3"/>
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" s="10">
+        <v>4</v>
+      </c>
+      <c r="C9" s="10">
+        <v>180</v>
+      </c>
+      <c r="D9" s="10">
+        <v>79</v>
+      </c>
+      <c r="E9" s="10">
+        <f t="shared" si="0"/>
+        <v>15.8</v>
+      </c>
+      <c r="F9" s="11">
+        <f t="shared" si="4"/>
+        <v>11.39240506329114</v>
+      </c>
+      <c r="G9" s="12">
+        <f t="shared" si="1"/>
+        <v>1501</v>
+      </c>
+      <c r="H9" s="13">
+        <f t="shared" si="2"/>
+        <v>1915.6666666666665</v>
+      </c>
+      <c r="I9" s="13">
+        <f t="shared" si="5"/>
+        <v>3416.6666666666665</v>
+      </c>
+      <c r="J9" s="13">
+        <f t="shared" si="3"/>
+        <v>1915.6666666666665</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" s="10">
+        <v>5</v>
+      </c>
+      <c r="C10" s="10">
+        <v>90</v>
+      </c>
+      <c r="D10" s="10">
+        <v>63</v>
+      </c>
+      <c r="E10" s="10">
+        <f t="shared" si="0"/>
+        <v>12.600000000000001</v>
+      </c>
+      <c r="F10" s="11">
+        <f t="shared" si="4"/>
+        <v>7.1428571428571423</v>
+      </c>
+      <c r="G10" s="12">
+        <f t="shared" si="1"/>
+        <v>1197</v>
+      </c>
+      <c r="H10" s="13">
+        <f t="shared" si="2"/>
+        <v>903.00000000000011</v>
+      </c>
+      <c r="I10" s="13">
+        <f t="shared" si="5"/>
+        <v>2100</v>
+      </c>
+      <c r="J10" s="13">
+        <f t="shared" si="3"/>
+        <v>1197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" s="10">
+        <v>5</v>
+      </c>
+      <c r="C11" s="10">
+        <v>120</v>
+      </c>
+      <c r="D11" s="10">
+        <v>93</v>
+      </c>
+      <c r="E11" s="10">
+        <f t="shared" si="0"/>
+        <v>18.600000000000001</v>
+      </c>
+      <c r="F11" s="11">
+        <f t="shared" si="4"/>
+        <v>6.4516129032258061</v>
+      </c>
+      <c r="G11" s="12">
+        <f t="shared" si="1"/>
+        <v>1767</v>
+      </c>
+      <c r="H11" s="13">
+        <f t="shared" si="2"/>
+        <v>1183</v>
+      </c>
+      <c r="I11" s="13">
+        <f t="shared" si="5"/>
+        <v>2950</v>
+      </c>
+      <c r="J11" s="13">
+        <f t="shared" si="3"/>
+        <v>1767</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12">
+        <v>1</v>
+      </c>
+      <c r="B12" s="10">
+        <v>1</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="12"/>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" s="10">
+        <v>2</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" s="10">
+        <v>3</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15" s="10">
+        <v>4</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16" s="10">
+        <v>5</v>
+      </c>
+      <c r="E16" s="8"/>
+      <c r="I16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="5:5">
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="5:5">
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="5:5">
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="5:5">
+      <c r="E24" s="1"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2:G11">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H11">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I11">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE46B-0EE8-4D7E-956E-06AD6DDE4FF5}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <cols>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" t="s">
-        <v>1</v>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="I6" s="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A48C4B-C23A-0343-9CD4-B20C0FE9227B}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
-    <col min="3" max="3" width="12.5" customWidth="1"/>
-    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <cols>
+    <col min="3" max="3" width="22.5" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1943,13 +2706,10 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1962,14 +2722,11 @@
       <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1982,14 +2739,11 @@
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1997,19 +2751,16 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="F4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -2017,19 +2768,16 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="F5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -2037,17 +2785,20 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="F6" t="s">
         <v>14</v>
       </c>
+    </row>
+    <row r="18" spans="4:5">
+      <c r="E18" s="6"/>
+    </row>
+    <row r="20" spans="4:5">
+      <c r="D20" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2055,16 +2806,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A73ABDEA-DD83-4C31-B1A2-B93032C8B1F1}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
   <dimension ref="A1:X32"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -2083,23 +2834,19 @@
       <c r="F1" t="s">
         <v>20</v>
       </c>
-      <c r="I1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
       <c r="D2">
-        <f ca="1">RANDBETWEEN(10,120)</f>
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -2107,32 +2854,19 @@
       <c r="F2">
         <v>1</v>
       </c>
-      <c r="I2">
-        <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>4</v>
-      </c>
-      <c r="K2">
-        <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D21" ca="1" si="0">RANDBETWEEN(10,120)</f>
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -2140,20 +2874,8 @@
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="I3">
-        <f t="shared" ref="I3:I21" ca="1" si="1">RANDBETWEEN(1,5)</f>
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <f t="shared" ref="K3:L21" ca="1" si="2">RANDBETWEEN(1,5)</f>
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <f t="shared" ca="1" si="2"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2161,11 +2883,10 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4">
-        <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -2173,20 +2894,8 @@
       <c r="F4">
         <v>0</v>
       </c>
-      <c r="I4">
-        <f t="shared" ca="1" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2197,8 +2906,7 @@
         <v>3</v>
       </c>
       <c r="D5">
-        <f t="shared" ca="1" si="0"/>
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -2206,32 +2914,19 @@
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="I5">
-        <f t="shared" ca="1" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <f t="shared" ca="1" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <f t="shared" ca="1" si="0"/>
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2239,32 +2934,19 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="I6">
-        <f t="shared" ca="1" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <f t="shared" ca="1" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <f t="shared" ca="1" si="0"/>
-        <v>118</v>
+        <v>35</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2272,32 +2954,19 @@
       <c r="F7">
         <v>1</v>
       </c>
-      <c r="I7">
-        <f t="shared" ca="1" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8">
         <v>3</v>
       </c>
       <c r="D8">
-        <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2305,32 +2974,19 @@
       <c r="F8">
         <v>1</v>
       </c>
-      <c r="I8">
-        <f t="shared" ca="1" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="K8">
-        <f t="shared" ca="1" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="L8">
-        <f t="shared" ca="1" si="2"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9">
-        <f t="shared" ca="1" si="0"/>
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -2338,32 +2994,19 @@
       <c r="F9">
         <v>1</v>
       </c>
-      <c r="I9">
-        <f t="shared" ca="1" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="K9">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L9">
-        <f t="shared" ca="1" si="2"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10">
-        <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -2371,32 +3014,19 @@
       <c r="F10">
         <v>0</v>
       </c>
-      <c r="I10">
-        <f t="shared" ca="1" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="K10">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="L10">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C11">
         <v>4</v>
       </c>
       <c r="D11">
-        <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2404,32 +3034,19 @@
       <c r="F11">
         <v>1</v>
       </c>
-      <c r="I11">
-        <f t="shared" ca="1" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="K11">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L11">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
       <c r="D12">
-        <f t="shared" ca="1" si="0"/>
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2437,32 +3054,19 @@
       <c r="F12">
         <v>0</v>
       </c>
-      <c r="I12">
-        <f t="shared" ca="1" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K12">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L12">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -2470,32 +3074,19 @@
       <c r="F13">
         <v>1</v>
       </c>
-      <c r="I13">
-        <f t="shared" ca="1" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="K13">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L13">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14">
-        <f t="shared" ca="1" si="0"/>
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -2503,32 +3094,19 @@
       <c r="F14">
         <v>1</v>
       </c>
-      <c r="I14">
-        <f t="shared" ca="1" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="K14">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L14">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D15">
-        <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2536,50 +3114,25 @@
       <c r="F15">
         <v>0</v>
       </c>
-      <c r="I15">
-        <f t="shared" ca="1" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="K15">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L15">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D16">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="E16">
         <v>3</v>
       </c>
       <c r="F16">
         <v>0</v>
-      </c>
-      <c r="I16">
-        <f t="shared" ca="1" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="K16">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="L16">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:24">
@@ -2587,32 +3140,19 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D17">
-        <f t="shared" ca="1" si="0"/>
-        <v>102</v>
+        <v>20</v>
       </c>
       <c r="E17">
         <v>3</v>
       </c>
       <c r="F17">
         <v>1</v>
-      </c>
-      <c r="I17">
-        <f t="shared" ca="1" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="K17">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="L17">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -2620,32 +3160,19 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18">
         <v>0</v>
-      </c>
-      <c r="I18">
-        <f t="shared" ca="1" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="K18">
-        <f t="shared" ca="1" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="L18">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -2653,32 +3180,19 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D19">
-        <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19">
         <v>0</v>
-      </c>
-      <c r="I19">
-        <f t="shared" ca="1" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="K19">
-        <f t="shared" ca="1" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="L19">
-        <f t="shared" ca="1" si="2"/>
-        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:24">
@@ -2686,32 +3200,19 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D20">
-        <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20">
         <v>0</v>
-      </c>
-      <c r="I20">
-        <f t="shared" ca="1" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K20">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="L20">
-        <f t="shared" ca="1" si="2"/>
-        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:24">
@@ -2719,32 +3220,19 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D21">
-        <f t="shared" ca="1" si="0"/>
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="F21">
         <v>0</v>
-      </c>
-      <c r="I21">
-        <f t="shared" ca="1" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="K21">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="L21">
-        <f t="shared" ca="1" si="2"/>
-        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:24">
@@ -2884,4 +3372,286 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF01B7F4-A8F2-E74F-93E1-1ACB4B99B891}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>45</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>80</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4154E97-9715-C248-8300-688A466787B4}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <cols>
+    <col min="3" max="3" width="12.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="I6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <cols>
+    <col min="3" max="3" width="12.5" customWidth="1"/>
+    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>